<commit_message>
Deploying to main from @ open-resource-discovery/specification@9f278ae95faabbf4a509721e62335779ae9c65c8 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-201/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-201/spec-v1/interfaces/Document.xlsx
@@ -391,10 +391,10 @@
     <t>target</t>
   </si>
   <si>
-    <t>OverlayTarget</t>
-  </si>
-  <si>
-    <t>Overlay Target</t>
+    <t>OverlayDefinitionTarget</t>
+  </si>
+  <si>
+    <t>Overlay Definition Target</t>
   </si>
   <si>
     <t>definitionType</t>

</xml_diff>

<commit_message>
Deploying to main from @ open-resource-discovery/specification@2d80b2c2bd40129b7e21f495536fa14fa2060091 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-201/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-201/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1444" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="212">
   <si>
     <t>Entity Name</t>
   </si>
@@ -398,6 +398,12 @@
   </si>
   <si>
     <t>definitionType</t>
+  </si>
+  <si>
+    <t>definitionPurpose</t>
+  </si>
+  <si>
+    <t>definitionVisibility</t>
   </si>
   <si>
     <t>Product</t>
@@ -1017,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D481"/>
+  <dimension ref="A1:D482"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4945,13 +4951,13 @@
         <v>127</v>
       </c>
       <c r="B281" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="C281" t="b">
         <v>0</v>
       </c>
       <c r="D281" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
@@ -4959,13 +4965,13 @@
         <v>127</v>
       </c>
       <c r="B282" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="C282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D282" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
@@ -4973,7 +4979,7 @@
         <v>127</v>
       </c>
       <c r="B283" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C283" t="b">
         <v>0</v>
@@ -4984,13 +4990,13 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B284" t="s">
-        <v>5</v>
+        <v>130</v>
       </c>
       <c r="C284" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D284" t="s">
         <v>6</v>
@@ -4998,38 +5004,38 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B285" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C285" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D285" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B286" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C286" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D286" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B287" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C287" t="b">
         <v>1</v>
@@ -5040,13 +5046,13 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B288" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C288" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D288" t="s">
         <v>6</v>
@@ -5054,13 +5060,13 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B289" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C289" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D289" t="s">
         <v>6</v>
@@ -5068,13 +5074,13 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B290" t="s">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="C290" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D290" t="s">
         <v>6</v>
@@ -5082,44 +5088,44 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B291" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
       <c r="C291" t="b">
         <v>0</v>
       </c>
       <c r="D291" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B292" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C292" t="b">
         <v>0</v>
       </c>
       <c r="D292" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B293" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C293" t="b">
         <v>0</v>
       </c>
       <c r="D293" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
@@ -5127,24 +5133,24 @@
         <v>131</v>
       </c>
       <c r="B294" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C294" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D294" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B295" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C295" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D295" t="s">
         <v>6</v>
@@ -5152,41 +5158,41 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B296" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C296" t="b">
         <v>0</v>
       </c>
       <c r="D296" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B297" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="C297" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D297" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B298" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C298" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D298" t="s">
         <v>6</v>
@@ -5194,13 +5200,13 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B299" t="s">
-        <v>10</v>
+        <v>115</v>
       </c>
       <c r="C299" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D299" t="s">
         <v>6</v>
@@ -5208,13 +5214,13 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B300" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C300" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D300" t="s">
         <v>6</v>
@@ -5222,10 +5228,10 @@
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B301" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C301" t="b">
         <v>0</v>
@@ -5236,10 +5242,10 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B302" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C302" t="b">
         <v>0</v>
@@ -5250,13 +5256,13 @@
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B303" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" t="s">
         <v>6</v>
@@ -5264,41 +5270,41 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B304" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C304" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D304" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B305" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C305" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D305" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B306" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C306" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D306" t="s">
         <v>6</v>
@@ -5306,13 +5312,13 @@
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B307" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C307" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D307" t="s">
         <v>6</v>
@@ -5320,10 +5326,10 @@
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B308" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C308" t="b">
         <v>1</v>
@@ -5334,195 +5340,195 @@
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B309" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C309" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D309" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B310" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B311" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B312" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B313" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B314" t="s">
-        <v>132</v>
+        <v>57</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B315" t="s">
-        <v>94</v>
+        <v>134</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B316" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>20</v>
+        <v>136</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B317" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B318" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B319" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B320" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="C320" t="b">
         <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B321" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C321" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B322" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C322" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D322" t="s">
         <v>6</v>
@@ -5530,13 +5536,13 @@
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B323" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C323" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D323" t="s">
         <v>6</v>
@@ -5544,10 +5550,10 @@
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B324" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C324" t="b">
         <v>1</v>
@@ -5558,38 +5564,38 @@
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B325" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C325" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D325" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B326" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B327" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
@@ -5600,13 +5606,13 @@
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B328" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="C328" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D328" t="s">
         <v>6</v>
@@ -5614,13 +5620,13 @@
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B329" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5628,41 +5634,41 @@
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B330" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C330" t="b">
         <v>0</v>
       </c>
       <c r="D330" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B331" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C331" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D331" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B332" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C332" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D332" t="s">
         <v>6</v>
@@ -5670,10 +5676,10 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B333" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C333" t="b">
         <v>0</v>
@@ -5684,13 +5690,13 @@
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B334" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="s">
         <v>6</v>
@@ -5698,41 +5704,41 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B335" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C335" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D335" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B336" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C336" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D336" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B337" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C337" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D337" t="s">
         <v>6</v>
@@ -5740,13 +5746,13 @@
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B338" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
         <v>6</v>
@@ -5754,10 +5760,10 @@
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B339" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C339" t="b">
         <v>1</v>
@@ -5768,13 +5774,13 @@
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B340" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C340" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D340" t="s">
         <v>6</v>
@@ -5782,49 +5788,49 @@
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B341" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B342" t="s">
-        <v>137</v>
+        <v>61</v>
       </c>
       <c r="C342" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D342" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B343" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D343" t="s">
-        <v>139</v>
+        <v>51</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B344" t="s">
         <v>140</v>
@@ -5833,88 +5839,88 @@
         <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>9</v>
+        <v>141</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B345" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="C345" t="b">
         <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B346" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C346" t="b">
         <v>0</v>
       </c>
       <c r="D346" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B347" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C347" t="b">
         <v>0</v>
       </c>
       <c r="D347" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B348" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C348" t="b">
         <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B349" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C349" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B350" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C350" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D350" t="s">
         <v>6</v>
@@ -5922,27 +5928,27 @@
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B351" t="s">
-        <v>137</v>
+        <v>12</v>
       </c>
       <c r="C351" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B352" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C352" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D352" t="s">
         <v>51</v>
@@ -5950,21 +5956,21 @@
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B353" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>144</v>
+        <v>51</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B354" t="s">
         <v>145</v>
@@ -5978,7 +5984,7 @@
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B355" t="s">
         <v>147</v>
@@ -5992,41 +5998,41 @@
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B356" t="s">
-        <v>32</v>
+        <v>149</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>33</v>
+        <v>150</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B357" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C357" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B358" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D358" t="s">
         <v>6</v>
@@ -6034,55 +6040,55 @@
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B359" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>152</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B360" t="s">
-        <v>32</v>
+        <v>153</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>33</v>
+        <v>154</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B361" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C361" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B362" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C362" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D362" t="s">
         <v>6</v>
@@ -6090,58 +6096,58 @@
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B363" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C363" t="b">
         <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
+        <v>155</v>
+      </c>
+      <c r="B364" t="s">
         <v>153</v>
       </c>
-      <c r="B364" t="s">
-        <v>155</v>
-      </c>
       <c r="C364" t="b">
         <v>0</v>
       </c>
       <c r="D364" t="s">
-        <v>9</v>
+        <v>156</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B365" t="s">
-        <v>32</v>
+        <v>157</v>
       </c>
       <c r="C365" t="b">
         <v>0</v>
       </c>
       <c r="D365" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B366" t="s">
-        <v>157</v>
+        <v>32</v>
       </c>
       <c r="C366" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
@@ -6163,7 +6169,7 @@
         <v>160</v>
       </c>
       <c r="B368" t="s">
-        <v>5</v>
+        <v>161</v>
       </c>
       <c r="C368" t="b">
         <v>1</v>
@@ -6174,13 +6180,13 @@
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B369" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D369" t="s">
         <v>6</v>
@@ -6188,38 +6194,38 @@
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B370" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="C370" t="b">
         <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B371" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C371" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B372" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C372" t="b">
         <v>1</v>
@@ -6230,24 +6236,24 @@
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B373" t="s">
-        <v>162</v>
+        <v>10</v>
       </c>
       <c r="C373" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D373" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B374" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="C374" t="b">
         <v>0</v>
@@ -6258,30 +6264,30 @@
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B375" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C375" t="b">
         <v>0</v>
       </c>
       <c r="D375" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B376" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C376" t="b">
         <v>0</v>
       </c>
       <c r="D376" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
@@ -6289,21 +6295,21 @@
         <v>163</v>
       </c>
       <c r="B377" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C377" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D377" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B378" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C378" t="b">
         <v>1</v>
@@ -6314,10 +6320,10 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B379" t="s">
-        <v>164</v>
+        <v>52</v>
       </c>
       <c r="C379" t="b">
         <v>1</v>
@@ -6328,13 +6334,13 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B380" t="s">
-        <v>12</v>
+        <v>166</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380" t="s">
         <v>6</v>
@@ -6342,10 +6348,10 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B381" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C381" t="b">
         <v>0</v>
@@ -6359,10 +6365,10 @@
         <v>165</v>
       </c>
       <c r="B382" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
         <v>6</v>
@@ -6370,10 +6376,10 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B383" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C383" t="b">
         <v>1</v>
@@ -6384,13 +6390,13 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B384" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D384" t="s">
         <v>6</v>
@@ -6398,13 +6404,13 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B385" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="s">
         <v>6</v>
@@ -6412,10 +6418,10 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B386" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C386" t="b">
         <v>1</v>
@@ -6426,13 +6432,13 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B387" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D387" t="s">
         <v>6</v>
@@ -6440,13 +6446,13 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B388" t="s">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="s">
         <v>6</v>
@@ -6454,10 +6460,10 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B389" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C389" t="b">
         <v>1</v>
@@ -6468,13 +6474,13 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B390" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C390" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D390" t="s">
         <v>6</v>
@@ -6482,13 +6488,13 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B391" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" t="s">
         <v>6</v>
@@ -6496,10 +6502,10 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B392" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6510,13 +6516,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B393" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6524,13 +6530,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B394" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C394" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6538,10 +6544,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B395" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C395" t="b">
         <v>1</v>
@@ -6552,13 +6558,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B396" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6566,13 +6572,13 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B397" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C397" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D397" t="s">
         <v>6</v>
@@ -6580,13 +6586,13 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B398" t="s">
-        <v>171</v>
+        <v>99</v>
       </c>
       <c r="C398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D398" t="s">
         <v>6</v>
@@ -6594,10 +6600,10 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B399" t="s">
-        <v>7</v>
+        <v>173</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
@@ -6608,58 +6614,58 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B400" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B401" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C401" t="b">
         <v>0</v>
       </c>
       <c r="D401" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B402" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
       </c>
       <c r="D402" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B403" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
@@ -6667,69 +6673,69 @@
         <v>172</v>
       </c>
       <c r="B404" t="s">
-        <v>173</v>
+        <v>31</v>
       </c>
       <c r="C404" t="b">
         <v>0</v>
       </c>
       <c r="D404" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B405" t="s">
-        <v>8</v>
+        <v>175</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B406" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B407" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B408" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
@@ -6737,21 +6743,21 @@
         <v>174</v>
       </c>
       <c r="B409" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B410" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
@@ -6762,83 +6768,83 @@
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B411" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B412" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B413" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B414" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B415" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C415" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B416" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C416" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D416" t="s">
         <v>6</v>
@@ -6846,10 +6852,10 @@
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B417" t="s">
-        <v>176</v>
+        <v>115</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
@@ -6863,10 +6869,10 @@
         <v>177</v>
       </c>
       <c r="B418" t="s">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="C418" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D418" t="s">
         <v>6</v>
@@ -6874,13 +6880,13 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B419" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C419" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6888,10 +6894,10 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B420" t="s">
-        <v>176</v>
+        <v>115</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
@@ -6902,7 +6908,7 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B421" t="s">
         <v>178</v>
@@ -6922,7 +6928,7 @@
         <v>180</v>
       </c>
       <c r="C422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="s">
         <v>6</v>
@@ -6930,10 +6936,10 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B423" t="s">
-        <v>10</v>
+        <v>182</v>
       </c>
       <c r="C423" t="b">
         <v>1</v>
@@ -6944,13 +6950,13 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B424" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C424" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D424" t="s">
         <v>6</v>
@@ -6958,38 +6964,38 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B425" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B426" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B427" t="s">
-        <v>181</v>
+        <v>8</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
@@ -7000,27 +7006,27 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B428" t="s">
-        <v>38</v>
+        <v>183</v>
       </c>
       <c r="C428" t="b">
         <v>0</v>
       </c>
       <c r="D428" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B429" t="s">
-        <v>183</v>
+        <v>38</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7028,10 +7034,10 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B430" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C430" t="b">
         <v>1</v>
@@ -7042,10 +7048,10 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
+        <v>184</v>
+      </c>
+      <c r="B431" t="s">
         <v>182</v>
-      </c>
-      <c r="B431" t="s">
-        <v>10</v>
       </c>
       <c r="C431" t="b">
         <v>1</v>
@@ -7056,13 +7062,13 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B432" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
         <v>6</v>
@@ -7070,38 +7076,38 @@
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B433" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B434" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B435" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
@@ -7112,27 +7118,27 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B436" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C436" t="b">
         <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="B437" t="s">
-        <v>184</v>
+        <v>38</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
         <v>6</v>
@@ -7143,10 +7149,10 @@
         <v>84</v>
       </c>
       <c r="B438" t="s">
-        <v>12</v>
+        <v>186</v>
       </c>
       <c r="C438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
         <v>6</v>
@@ -7154,27 +7160,27 @@
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>185</v>
+        <v>84</v>
       </c>
       <c r="B439" t="s">
-        <v>186</v>
+        <v>12</v>
       </c>
       <c r="C439" t="b">
         <v>0</v>
       </c>
       <c r="D439" t="s">
-        <v>187</v>
+        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B440" t="s">
         <v>188</v>
       </c>
       <c r="C440" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D440" t="s">
         <v>189</v>
@@ -7182,24 +7188,24 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
+        <v>187</v>
+      </c>
+      <c r="B441" t="s">
         <v>190</v>
       </c>
-      <c r="B441" t="s">
-        <v>5</v>
-      </c>
       <c r="C441" t="b">
         <v>1</v>
       </c>
       <c r="D441" t="s">
-        <v>6</v>
+        <v>191</v>
       </c>
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B442" t="s">
-        <v>191</v>
+        <v>5</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7213,7 +7219,7 @@
         <v>192</v>
       </c>
       <c r="B443" t="s">
-        <v>5</v>
+        <v>193</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7224,10 +7230,10 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B444" t="s">
-        <v>191</v>
+        <v>5</v>
       </c>
       <c r="C444" t="b">
         <v>1</v>
@@ -7238,10 +7244,10 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
+        <v>194</v>
+      </c>
+      <c r="B445" t="s">
         <v>193</v>
-      </c>
-      <c r="B445" t="s">
-        <v>97</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7252,10 +7258,10 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B446" t="s">
-        <v>194</v>
+        <v>97</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7269,7 +7275,7 @@
         <v>195</v>
       </c>
       <c r="B447" t="s">
-        <v>97</v>
+        <v>196</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7280,10 +7286,10 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B448" t="s">
-        <v>196</v>
+        <v>97</v>
       </c>
       <c r="C448" t="b">
         <v>1</v>
@@ -7297,7 +7303,7 @@
         <v>197</v>
       </c>
       <c r="B449" t="s">
-        <v>5</v>
+        <v>198</v>
       </c>
       <c r="C449" t="b">
         <v>1</v>
@@ -7308,7 +7314,7 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B450" t="s">
         <v>5</v>
@@ -7322,10 +7328,10 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B451" t="s">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="C451" t="b">
         <v>1</v>
@@ -7339,7 +7345,7 @@
         <v>201</v>
       </c>
       <c r="B452" t="s">
-        <v>5</v>
+        <v>202</v>
       </c>
       <c r="C452" t="b">
         <v>1</v>
@@ -7350,13 +7356,13 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B453" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C453" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D453" t="s">
         <v>6</v>
@@ -7367,10 +7373,10 @@
         <v>203</v>
       </c>
       <c r="B454" t="s">
-        <v>5</v>
+        <v>204</v>
       </c>
       <c r="C454" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D454" t="s">
         <v>6</v>
@@ -7378,13 +7384,13 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B455" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C455" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D455" t="s">
         <v>6</v>
@@ -7392,13 +7398,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
+        <v>205</v>
+      </c>
+      <c r="B456" t="s">
         <v>204</v>
       </c>
-      <c r="B456" t="s">
-        <v>5</v>
-      </c>
       <c r="C456" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7406,13 +7412,13 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B457" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C457" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D457" t="s">
         <v>6</v>
@@ -7420,13 +7426,13 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B458" t="s">
-        <v>5</v>
+        <v>204</v>
       </c>
       <c r="C458" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D458" t="s">
         <v>6</v>
@@ -7434,13 +7440,13 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B459" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7448,13 +7454,13 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B460" t="s">
-        <v>5</v>
+        <v>204</v>
       </c>
       <c r="C460" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D460" t="s">
         <v>6</v>
@@ -7462,13 +7468,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B461" t="s">
         <v>5</v>
       </c>
       <c r="C461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7476,10 +7482,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B462" t="s">
-        <v>183</v>
+        <v>5</v>
       </c>
       <c r="C462" t="b">
         <v>0</v>
@@ -7490,10 +7496,10 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B463" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C463" t="b">
         <v>0</v>
@@ -7504,13 +7510,13 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B464" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="C464" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D464" t="s">
         <v>6</v>
@@ -7518,13 +7524,13 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B465" t="s">
-        <v>12</v>
+        <v>210</v>
       </c>
       <c r="C465" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D465" t="s">
         <v>6</v>
@@ -7535,10 +7541,10 @@
         <v>209</v>
       </c>
       <c r="B466" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7546,13 +7552,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B467" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7560,41 +7566,41 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B468" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C468" t="b">
         <v>0</v>
       </c>
       <c r="D468" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B469" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B470" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7602,13 +7608,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B471" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7616,10 +7622,10 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B472" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C472" t="b">
         <v>1</v>
@@ -7630,41 +7636,41 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B473" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C473" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D473" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B474" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C474" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D474" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B475" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C475" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D475" t="s">
         <v>6</v>
@@ -7672,13 +7678,13 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B476" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C476" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7686,10 +7692,10 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B477" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C477" t="b">
         <v>1</v>
@@ -7700,57 +7706,71 @@
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B478" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C478" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D478" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B479" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
       </c>
       <c r="D479" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B480" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C480" t="b">
         <v>0</v>
       </c>
       <c r="D480" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B481" t="s">
+        <v>32</v>
+      </c>
+      <c r="C481" t="b">
+        <v>0</v>
+      </c>
+      <c r="D481" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>211</v>
+      </c>
+      <c r="B482" t="s">
         <v>34</v>
       </c>
-      <c r="C481" t="b">
-        <v>0</v>
-      </c>
-      <c r="D481" t="s">
+      <c r="C482" t="b">
+        <v>0</v>
+      </c>
+      <c r="D482" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>